<commit_message>
correccion de lineas verticales en el grafico de historico de acciones
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{729736CF-31FF-4164-94AA-912E95DCB7CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062D0FF8-36C8-4608-BBD7-B445F9C51FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4380" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -36,10 +36,19 @@
     <t>Implementar dashboard con indicadores</t>
   </si>
   <si>
-    <t>Corregir la contabilidad con los movimientos</t>
-  </si>
-  <si>
     <t>Añadir funcionalidad relacionada con el registro de las utilidades por otro tipo de transacciones - venta bonos - venta acciones - venta notas credito</t>
+  </si>
+  <si>
+    <t>Corregir error de calculo en la generación de amortizacion</t>
+  </si>
+  <si>
+    <t>Registrar las ganancias por otras actividades como venta de acciones</t>
+  </si>
+  <si>
+    <t>Registrar las ganancias por otras actividades como venta de notas de crédito</t>
+  </si>
+  <si>
+    <t>Corregir la contabilidad con los movimientos - ahortia toma información de la tabla de inversiones</t>
   </si>
 </sst>
 </file>
@@ -357,7 +366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:B6"/>
+  <dimension ref="B2:B9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="105" customWidth="1"/>
@@ -380,12 +389,27 @@
     </row>
     <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se añaden lineas verticales en el grafico de año particular
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062D0FF8-36C8-4608-BBD7-B445F9C51FD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597BB124-7F6D-41FE-B256-DBC2C2EDCB11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4380" yWindow="3855" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$10</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -49,14 +52,64 @@
   </si>
   <si>
     <t>Corregir la contabilidad con los movimientos - ahortia toma información de la tabla de inversiones</t>
+  </si>
+  <si>
+    <t>Grafico solapado de los precios de las acciones de todos los años para poder visualizar comportamiento ciclico de las acciones de una empresa</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>Módulo</t>
+  </si>
+  <si>
+    <t>Descripción</t>
+  </si>
+  <si>
+    <t>Prioridad</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Registro</t>
+  </si>
+  <si>
+    <t>Finalizado</t>
+  </si>
+  <si>
+    <t>Acciones</t>
+  </si>
+  <si>
+    <t>Dashboard</t>
+  </si>
+  <si>
+    <t>Contabilidad</t>
+  </si>
+  <si>
+    <t>Utilidades</t>
+  </si>
+  <si>
+    <t>Amortizaciones</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -84,8 +137,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -366,53 +421,229 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:B9"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="105" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="133.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
       <c r="B2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
       <c r="B3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
       <c r="B5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
       <c r="B6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
       <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
       <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
       <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
         <v>6</v>
       </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="2">
+        <v>46193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="2">
+        <v>46193</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G10" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Primera version del dashboard de acciones propias
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597BB124-7F6D-41FE-B256-DBC2C2EDCB11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58DC410-DA45-4F2D-91D5-84FCC9667EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$11</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="25">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -51,9 +51,6 @@
     <t>Registrar las ganancias por otras actividades como venta de notas de crédito</t>
   </si>
   <si>
-    <t>Corregir la contabilidad con los movimientos - ahortia toma información de la tabla de inversiones</t>
-  </si>
-  <si>
     <t>Grafico solapado de los precios de las acciones de todos los años para poder visualizar comportamiento ciclico de las acciones de una empresa</t>
   </si>
   <si>
@@ -94,6 +91,18 @@
   </si>
   <si>
     <t>Pendiente</t>
+  </si>
+  <si>
+    <t>Listo</t>
+  </si>
+  <si>
+    <t>Implementar la lectura de archivos PDF desde el mismo sistema para carga de notas de crédito</t>
+  </si>
+  <si>
+    <t>Corregir la contabilidad con los movimientos - ahorita toma información de la tabla de inversiones</t>
+  </si>
+  <si>
+    <t>Notas Credito</t>
   </si>
 </sst>
 </file>
@@ -422,10 +431,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="133.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
@@ -435,25 +444,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -461,7 +470,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C2" t="s">
         <v>0</v>
@@ -474,6 +483,9 @@
       </c>
       <c r="F2" s="2">
         <v>46193</v>
+      </c>
+      <c r="G2" s="2">
+        <v>46194</v>
       </c>
     </row>
     <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -481,7 +493,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -490,7 +502,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F3" s="2">
         <v>46193</v>
@@ -501,7 +513,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
@@ -510,7 +522,7 @@
         <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" s="2">
         <v>46193</v>
@@ -521,16 +533,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F5" s="2">
         <v>46193</v>
@@ -541,7 +553,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
         <v>3</v>
@@ -550,7 +562,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" s="2">
         <v>46193</v>
@@ -561,7 +573,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
         <v>4</v>
@@ -570,7 +582,7 @@
         <v>1</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F7" s="2">
         <v>46193</v>
@@ -581,7 +593,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" t="s">
         <v>5</v>
@@ -590,7 +602,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F8" s="2">
         <v>46193</v>
@@ -601,7 +613,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
         <v>6</v>
@@ -610,7 +622,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F9" s="2">
         <v>46193</v>
@@ -621,23 +633,43 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D10">
         <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F10" s="2">
         <v>46193</v>
       </c>
     </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="2">
+        <v>46194</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G10" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:G11" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="3">
       <filters>
         <filter val="1"/>

</xml_diff>

<commit_message>
Arreglos en la pantalla de Amortizacion
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D58DC410-DA45-4F2D-91D5-84FCC9667EC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4699C7E6-BBD9-4E5E-B993-685F63DCD6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>Notas Credito</t>
+  </si>
+  <si>
+    <t>Pedir documentacion de los parametros creados como se los debe utilizar</t>
   </si>
 </sst>
 </file>
@@ -431,7 +434,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -668,6 +671,11 @@
         <v>46194</v>
       </c>
     </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G11" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="3">

</xml_diff>

<commit_message>
Mejora en la pantalla de Venta de Notas de Crédito
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4699C7E6-BBD9-4E5E-B993-685F63DCD6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07251D5A-DDEE-4C96-83B4-830D80DA9A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -168,6 +168,143 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>895350</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>66675</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>597905</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>27556</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1983F9A5-4D29-E62E-1503-AD3012DDED06}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1095375" y="2162175"/>
+          <a:ext cx="17361905" cy="8152381"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>6638095</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>94643</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26FE1002-5B77-53A7-EB4F-D82A86DD0F6C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1181100" y="10668000"/>
+          <a:ext cx="6638095" cy="4857143"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>6686550</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>532618</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>75590</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C14DC80-896D-450A-A78F-5FAF431E2923}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7867650" y="10629900"/>
+          <a:ext cx="6257143" cy="4876190"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -685,5 +822,6 @@
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
La pantalla ahora considera el toggle con dividendo en acciones o no
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07251D5A-DDEE-4C96-83B4-830D80DA9A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A81910-EB80-4C1F-9564-2FC9055245FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Correccion en pantalla codigo_valor
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A81910-EB80-4C1F-9564-2FC9055245FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025A1872-6039-450F-AF73-A7AB01EB7506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="29">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -106,6 +106,15 @@
   </si>
   <si>
     <t>Pedir documentacion de los parametros creados como se los debe utilizar</t>
+  </si>
+  <si>
+    <t>Actualizar gráfico relacionado con ganancias por otro tipo de utilidades</t>
+  </si>
+  <si>
+    <t>Revisar el calculo de las utilidadespor venta de bonos, venta de acciones, venta de notas de crédito</t>
+  </si>
+  <si>
+    <t>Parametrizacion</t>
   </si>
 </sst>
 </file>
@@ -176,13 +185,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>895350</xdr:colOff>
-      <xdr:row>14</xdr:row>
+      <xdr:row>22</xdr:row>
       <xdr:rowOff>66675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>597905</xdr:colOff>
-      <xdr:row>57</xdr:row>
+      <xdr:row>65</xdr:row>
       <xdr:rowOff>27556</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -220,13 +229,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:row>67</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>6638095</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>92</xdr:row>
       <xdr:rowOff>94643</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -264,13 +273,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>6686550</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>66</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
       <xdr:colOff>532618</xdr:colOff>
-      <xdr:row>84</xdr:row>
+      <xdr:row>92</xdr:row>
       <xdr:rowOff>75590</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -571,7 +580,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -809,8 +818,54 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>28</v>
+      </c>
       <c r="C12" t="s">
         <v>25</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="2">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="2">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="2">
+        <v>46194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se elimina el premio de Vencimientos Semanales
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F882D022-F7F0-4B2D-B635-E58E76645045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A58717-FC8B-44DA-8FCA-EA2871FCB811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -126,10 +126,10 @@
     <t>Dividir en el excel Brikapital de las otras acciones</t>
   </si>
   <si>
-    <t>Validar si los ultimos bonos vendidos aparecen en el resumen de utiliades por ventas</t>
-  </si>
-  <si>
     <t>Implementar el dashboard con los mejores indicadores</t>
+  </si>
+  <si>
+    <t>Validar si los ultimos bonos vendidos aparecen en el resumen de utilidades por ventas</t>
   </si>
 </sst>
 </file>
@@ -562,7 +562,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D4" s="2">
         <v>2</v>
@@ -868,7 +868,7 @@
         <v>17</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D18" s="2">
         <v>1</v>

</xml_diff>

<commit_message>
Creacion de la la lista de venta de Notas de crédito
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A58717-FC8B-44DA-8FCA-EA2871FCB811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB09C5C1-6270-430C-BD6B-60E2BA6D8545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="35">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>Validar si los ultimos bonos vendidos aparecen en el resumen de utilidades por ventas</t>
+  </si>
+  <si>
+    <t>Revisar el listado de venta de notas de crédito</t>
   </si>
 </sst>
 </file>
@@ -188,11 +191,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -474,7 +478,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -892,6 +896,27 @@
       <c r="F19" s="3"/>
       <c r="G19" s="2"/>
     </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="4">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="2">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" s="3">
+        <v>46204</v>
+      </c>
+      <c r="G20" s="2"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G19" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">

</xml_diff>

<commit_message>
Exlusion notas creddito de Renta fija y adicion de detalle en las acciones compradas en el dia
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB09C5C1-6270-430C-BD6B-60E2BA6D8545}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB43AD72-5BE8-43A7-BC71-A21955266B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -132,7 +132,7 @@
     <t>Validar si los ultimos bonos vendidos aparecen en el resumen de utilidades por ventas</t>
   </si>
   <si>
-    <t>Revisar el listado de venta de notas de crédito</t>
+    <t>Revisar el listado de venta de notas de crédito - se debe validar de donde está saliendo la informacion, falta el valor nominal</t>
   </si>
 </sst>
 </file>
@@ -191,12 +191,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -897,13 +896,13 @@
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="4">
+      <c r="A20" s="2">
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="2" t="s">
         <v>34</v>
       </c>
       <c r="D20" s="2">

</xml_diff>

<commit_message>
Correcion en las vistas de notas de credito que se perdieron
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB43AD72-5BE8-43A7-BC71-A21955266B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBE5E72-D19C-4AAB-ABFF-0F612B4CB161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3150" yWindow="4515" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="36">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>Revisar el listado de venta de notas de crédito - se debe validar de donde está saliendo la informacion, falta el valor nominal</t>
+  </si>
+  <si>
+    <t>Actualizar archivo manual de acciones compradas</t>
   </si>
 </sst>
 </file>
@@ -164,7 +167,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -187,15 +190,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,7 +492,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -916,6 +931,23 @@
       </c>
       <c r="G20" s="2"/>
     </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="4">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D21" s="2">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G19" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">

</xml_diff>

<commit_message>
Eliminación de los campos activo y pagada de la tabla amortizacion. Tambien pequeñas mejoras en las pantallas de amortizacion
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CBE5E72-D19C-4AAB-ABFF-0F612B4CB161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1906E5B-1BC1-4EA6-9730-8A19626B55C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3150" yWindow="4515" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -136,6 +136,14 @@
   </si>
   <si>
     <t>Actualizar archivo manual de acciones compradas</t>
+  </si>
+  <si>
+    <t>Ventas</t>
+  </si>
+  <si>
+    <t>Parece que al migrar las ventas del archivo original, cargué el campo equivocado en el campo ganancia anual. Se debio cargar "% Ganancia Anual estimado", esta cargado "Tasa Anualizada" - actualizado manualmente en para notas de credito … falta actualizar para las otras ventas
+select fecha_venta, liquidacion_venta, ganancia_perdida, rendimiento_total, dias_transcurridos, roi, ganancia_anual from venta_inversion where id_tipo_venta = 195 order by fecha_venta
+select * from venta_inversion where id_tipo_venta = 195 order by fecha_venta</t>
   </si>
 </sst>
 </file>
@@ -167,7 +175,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -201,16 +209,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -492,12 +529,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="133.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="133.5703125" style="8" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
@@ -510,7 +547,7 @@
       <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -579,7 +616,7 @@
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="7" t="s">
         <v>32</v>
       </c>
       <c r="D4" s="2">
@@ -600,7 +637,7 @@
       <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="7" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="2">
@@ -644,7 +681,7 @@
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="7" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="2">
@@ -730,7 +767,7 @@
       <c r="B11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="7" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="2">
@@ -820,7 +857,7 @@
       <c r="B15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="7" t="s">
         <v>28</v>
       </c>
       <c r="D15" s="2">
@@ -864,7 +901,7 @@
       <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="7" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="2">
@@ -885,7 +922,7 @@
       <c r="B18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="7" t="s">
         <v>33</v>
       </c>
       <c r="D18" s="2">
@@ -903,12 +940,12 @@
       <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="2"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="9"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -917,7 +954,7 @@
       <c r="B20" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D20" s="2">
@@ -935,10 +972,10 @@
       <c r="A21" s="4">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="7" t="s">
         <v>35</v>
       </c>
       <c r="D21" s="2">
@@ -947,6 +984,31 @@
       <c r="E21" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="F21" s="3">
+        <v>46215</v>
+      </c>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>21</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F22" s="3">
+        <v>46215</v>
+      </c>
+      <c r="G22" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G19" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>

<commit_message>
Coreccion de errores en la pantalla Flujo de Capital
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1906E5B-1BC1-4EA6-9730-8A19626B55C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594AC38B-CA56-4D51-B991-8E1B89EB3AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="39">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -144,6 +144,9 @@
     <t>Parece que al migrar las ventas del archivo original, cargué el campo equivocado en el campo ganancia anual. Se debio cargar "% Ganancia Anual estimado", esta cargado "Tasa Anualizada" - actualizado manualmente en para notas de credito … falta actualizar para las otras ventas
 select fecha_venta, liquidacion_venta, ganancia_perdida, rendimiento_total, dias_transcurridos, roi, ganancia_anual from venta_inversion where id_tipo_venta = 195 order by fecha_venta
 select * from venta_inversion where id_tipo_venta = 195 order by fecha_venta</t>
+  </si>
+  <si>
+    <t>a ultranza</t>
   </si>
 </sst>
 </file>
@@ -226,13 +229,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -244,10 +246,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,12 +527,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="133.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="133.5703125" style="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
@@ -547,7 +545,7 @@
       <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -616,7 +614,7 @@
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>32</v>
       </c>
       <c r="D4" s="2">
@@ -637,7 +635,7 @@
       <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="2">
@@ -681,7 +679,7 @@
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="2">
@@ -767,7 +765,7 @@
       <c r="B11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="2">
@@ -857,7 +855,7 @@
       <c r="B15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="7" t="s">
+      <c r="C15" s="6" t="s">
         <v>28</v>
       </c>
       <c r="D15" s="2">
@@ -901,7 +899,7 @@
       <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="2">
@@ -922,7 +920,7 @@
       <c r="B18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="C18" s="6" t="s">
         <v>33</v>
       </c>
       <c r="D18" s="2">
@@ -940,12 +938,12 @@
       <c r="A19" s="2">
         <v>18</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="9"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="8"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
@@ -954,7 +952,7 @@
       <c r="B20" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="C20" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D20" s="2">
@@ -975,7 +973,7 @@
       <c r="B21" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="C21" s="6" t="s">
         <v>35</v>
       </c>
       <c r="D21" s="2">
@@ -990,13 +988,13 @@
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A22" s="5">
+      <c r="A22" s="4">
         <v>21</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="6" t="s">
         <v>37</v>
       </c>
       <c r="D22" s="2">
@@ -1009,6 +1007,11 @@
         <v>46215</v>
       </c>
       <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C23" s="7" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G19" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>

<commit_message>
Estandarizacion de estilos en las tablas y adición de calculo de dividendos en el calculo del patrimonio
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{594AC38B-CA56-4D51-B991-8E1B89EB3AB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED6D4162-776C-49A8-BC66-12F7933AC289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23805" yWindow="2145" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="40">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -147,6 +147,9 @@
   </si>
   <si>
     <t>a ultranza</t>
+  </si>
+  <si>
+    <t>En la tabla de Ventas no hay el campo valor nominal - entre "Fecha Venta" y "Precio Venta" añade valor nominal</t>
   </si>
 </sst>
 </file>
@@ -527,7 +530,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -1013,6 +1016,11 @@
         <v>38</v>
       </c>
     </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C24" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G19" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">

</xml_diff>

<commit_message>
Mejoras visuales en venta de Notas de Crédito
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED6D4162-776C-49A8-BC66-12F7933AC289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1FFCD9-E7CE-4779-9B85-67760B231439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23805" yWindow="2145" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Mejoras en las tarjetas de inversiones de renta variable
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA1FFCD9-E7CE-4779-9B85-67760B231439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE804ED8-24BB-4F82-A61E-2EF8DCD7DF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Actualizacion del Dashboard de Renta Variable
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE804ED8-24BB-4F82-A61E-2EF8DCD7DF7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D384040C-CB6A-4699-B8F9-8CE7869136E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="46">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -150,6 +150,24 @@
   </si>
   <si>
     <t>En la tabla de Ventas no hay el campo valor nominal - entre "Fecha Venta" y "Precio Venta" añade valor nominal</t>
+  </si>
+  <si>
+    <t>Como actuó al vender acciones?</t>
+  </si>
+  <si>
+    <t>Adicionalmente el porcentaje de las ventas parece que está mal</t>
+  </si>
+  <si>
+    <t>La imagen es para el 4 de agosto … la cantidad de transacciones esta mal … hubieron mas transacciones ese día …</t>
+  </si>
+  <si>
+    <t>en el gráfico solapado los puntos corresponden a distintas fechas</t>
+  </si>
+  <si>
+    <t>id_inversion</t>
+  </si>
+  <si>
+    <t>id_venta_inversion</t>
   </si>
 </sst>
 </file>
@@ -173,12 +191,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -232,7 +256,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -249,6 +273,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -264,6 +292,151 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1025" name="AutoShape 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{275299FC-8F7D-AA02-FF2F-F5590C4DC724}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1181100" y="4381500"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1026" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C84F955B-FE31-4790-B273-2F6834EAA456}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1181100" y="3619500"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>3857143</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>3661</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1453126-DB7F-FC19-2407-EF0E6205E0F6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1182121" y="3946071"/>
+          <a:ext cx="3857143" cy="3371429"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -530,13 +703,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="133.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -624,12 +797,14 @@
         <v>2</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4" s="3">
         <v>46193</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" s="3">
+        <v>46235</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -1019,6 +1194,76 @@
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C24" s="7" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C25" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C26" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C27" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E30">
+        <v>28401.05</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C31"/>
+      <c r="E31" s="11">
+        <v>28374.3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E32">
+        <f>E30-E31</f>
+        <v>26.75</v>
+      </c>
+    </row>
+    <row r="37" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E37" t="s">
+        <v>44</v>
+      </c>
+      <c r="F37">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="38" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E38" t="s">
+        <v>45</v>
+      </c>
+      <c r="F38">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="41" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E41">
+        <v>752.79</v>
+      </c>
+      <c r="F41">
+        <v>26.75</v>
+      </c>
+    </row>
+    <row r="42" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E42">
+        <v>100</v>
+      </c>
+      <c r="F42">
+        <f>E42*F41/E41</f>
+        <v>3.5534478406992656</v>
+      </c>
+    </row>
+    <row r="47" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C47" s="7" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1030,5 +1275,6 @@
     </filterColumn>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mejoras en modal de flujo de caja
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D384040C-CB6A-4699-B8F9-8CE7869136E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4FD8370-39EA-4F95-AFB6-D044C04C774A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="48">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -168,6 +168,12 @@
   </si>
   <si>
     <t>id_venta_inversion</t>
+  </si>
+  <si>
+    <t>Permitir actualizar la fecha de amortizacion desde flujo de capital</t>
+  </si>
+  <si>
+    <t>Crear opción para sacar el snapshot de todos los indicadores y luego sacar gráficos</t>
   </si>
 </sst>
 </file>
@@ -205,7 +211,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -228,40 +234,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -271,12 +252,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -403,7 +380,7 @@
       <xdr:col>2</xdr:col>
       <xdr:colOff>3857143</xdr:colOff>
       <xdr:row>46</xdr:row>
-      <xdr:rowOff>3661</xdr:rowOff>
+      <xdr:rowOff>3662</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -703,12 +680,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="133.5703125" style="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="133.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
@@ -721,7 +698,7 @@
       <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -783,14 +760,14 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D4" s="2">
@@ -813,7 +790,7 @@
       <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="2">
@@ -850,26 +827,28 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
         <v>3</v>
       </c>
       <c r="D7" s="2">
         <v>1</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F7" s="3">
         <v>46193</v>
       </c>
-      <c r="G7" s="2"/>
+      <c r="G7" s="3">
+        <v>46249</v>
+      </c>
     </row>
     <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -943,7 +922,7 @@
       <c r="B11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>21</v>
       </c>
       <c r="D11" s="2">
@@ -1026,26 +1005,28 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="5" t="s">
         <v>28</v>
       </c>
       <c r="D15" s="2">
         <v>1</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F15" s="3">
         <v>46204</v>
       </c>
-      <c r="G15" s="2"/>
+      <c r="G15" s="3">
+        <v>46249</v>
+      </c>
     </row>
     <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -1077,7 +1058,7 @@
       <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D17" s="2">
@@ -1098,7 +1079,7 @@
       <c r="B18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D18" s="2">
@@ -1114,45 +1095,59 @@
     </row>
     <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
-        <v>18</v>
-      </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="8"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="2">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="3">
+        <v>46204</v>
+      </c>
+      <c r="G19" s="3">
+        <v>46249</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>34</v>
+        <v>14</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="D20" s="2">
         <v>1</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F20" s="3">
-        <v>46204</v>
-      </c>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="4">
-        <v>20</v>
+        <v>46215</v>
+      </c>
+      <c r="G20" s="3">
+        <v>46249</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="D21" s="2">
         <v>1</v>
@@ -1161,19 +1156,19 @@
         <v>19</v>
       </c>
       <c r="F21" s="3">
-        <v>46215</v>
+        <v>46249</v>
       </c>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A22" s="4">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>37</v>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>22</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>47</v>
       </c>
       <c r="D22" s="2">
         <v>1</v>
@@ -1182,34 +1177,114 @@
         <v>19</v>
       </c>
       <c r="F22" s="3">
-        <v>46215</v>
+        <v>46249</v>
       </c>
       <c r="G22" s="2"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="7" t="s">
-        <v>38</v>
-      </c>
+      <c r="A23" s="2">
+        <v>23</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" s="2">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="3">
+        <v>46249</v>
+      </c>
+      <c r="G23" s="2"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C24" s="7" t="s">
+      <c r="A24" s="2">
+        <v>24</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>39</v>
       </c>
+      <c r="D24" s="2">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="3">
+        <v>46249</v>
+      </c>
+      <c r="G24" s="2"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C25" s="7" t="s">
+      <c r="A25" s="2">
+        <v>25</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>40</v>
       </c>
+      <c r="D25" s="2">
+        <v>1</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="3">
+        <v>46249</v>
+      </c>
+      <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C26" s="7" t="s">
+      <c r="A26" s="2">
+        <v>26</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>41</v>
       </c>
+      <c r="D26" s="2">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="3">
+        <v>46249</v>
+      </c>
+      <c r="G26" s="2"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C27" s="10" t="s">
+      <c r="A27" s="2">
+        <v>27</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>42</v>
       </c>
+      <c r="D27" s="2">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="3">
+        <v>46249</v>
+      </c>
+      <c r="G27" s="2"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="E30">
@@ -1218,7 +1293,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C31"/>
-      <c r="E31" s="11">
+      <c r="E31" s="7">
         <v>28374.3</v>
       </c>
     </row>
@@ -1262,14 +1337,19 @@
       </c>
     </row>
     <row r="47" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C47" s="7" t="s">
+      <c r="C47" s="6" t="s">
         <v>43</v>
       </c>
     </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C49" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G19" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <autoFilter ref="A1:G27" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="4">
-      <filters>
+      <filters blank="1">
         <filter val="Pendiente"/>
       </filters>
     </filterColumn>

</xml_diff>

<commit_message>
Mejoras en el Dashboard. Grabacion de indicadores en tabla historica
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4FD8370-39EA-4F95-AFB6-D044C04C774A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947AA1A2-5870-4CDF-BE5C-3AD5B35DCED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -238,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -253,7 +253,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -372,15 +371,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>68035</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>76541</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3857143</xdr:colOff>
-      <xdr:row>46</xdr:row>
-      <xdr:rowOff>3662</xdr:rowOff>
+      <xdr:colOff>3925178</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>80202</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -403,7 +402,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1182121" y="3946071"/>
+          <a:off x="1250156" y="3648416"/>
           <a:ext cx="3857143" cy="3371429"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1164,7 +1163,7 @@
       <c r="A22" s="2">
         <v>22</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C22" s="5" t="s">
@@ -1185,7 +1184,7 @@
       <c r="A23" s="2">
         <v>23</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C23" s="5" t="s">
@@ -1206,7 +1205,7 @@
       <c r="A24" s="2">
         <v>24</v>
       </c>
-      <c r="B24" s="8" t="s">
+      <c r="B24" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -1227,7 +1226,7 @@
       <c r="A25" s="2">
         <v>25</v>
       </c>
-      <c r="B25" s="8" t="s">
+      <c r="B25" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C25" s="5" t="s">
@@ -1248,7 +1247,7 @@
       <c r="A26" s="2">
         <v>26</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="2" t="s">
         <v>36</v>
       </c>
       <c r="C26" s="5" t="s">
@@ -1269,7 +1268,7 @@
       <c r="A27" s="2">
         <v>27</v>
       </c>
-      <c r="B27" s="8" t="s">
+      <c r="B27" s="2" t="s">
         <v>14</v>
       </c>
       <c r="C27" s="5" t="s">

</xml_diff>

<commit_message>
Implementac ion de nuevos graficos de tendencias
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{947AA1A2-5870-4CDF-BE5C-3AD5B35DCED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC92654-0AED-4DD8-92BC-34E30F2F5E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="57">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -174,13 +174,154 @@
   </si>
   <si>
     <t>Crear opción para sacar el snapshot de todos los indicadores y luego sacar gráficos</t>
+  </si>
+  <si>
+    <t>Preguntar que tipo de graficos se pueden sacar con la nueva información de Indicadores</t>
+  </si>
+  <si>
+    <r>
+      <t>1.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">       </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>¿En qué más podrías utilizar esta información histórica?</t>
+    </r>
+  </si>
+  <si>
+    <t>Además de crear gráficos de líneas o barras para ver la variación en el tiempo (que de por sí ya es muy valioso), tener este historial te abre la puerta a funcionalidades muy avanzadas:</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Cálculo de Crecimiento Porcentual (MoM / YoY):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> Podrás comparar automáticamente cuánto creció tu Patrimonio Consolidado o tus Intereses Esperados respecto al mes anterior (Month-over-Month) o al mismo mes del año pasado (Year-over-Year). Por ejemplo: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"Tu patrimonio creció un 4.5% este mes"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. Desviación de Proyecciones:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> Actualmente el sistema calcula tu "Proyección a 1 año". Si guardas el historial, podrás comparar si el crecimiento real de tu patrimonio cumplió con la proyección que habías hecho hace 1 año.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. Auditoría y Conciliación a Fin de Mes:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> Al tener una instantánea de cómo cerró tu portafolio el último día del mes, puedes usar ese registro exacto para conciliarlo contra tus estados de cuenta bancarios o de las casas de valores sin miedo a que una transacción ingresada tarde te mueva los números del pasado.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. Alertas de Caídas de Liquidez o Valor:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> Si el sistema detecta que tu "Total Corriente" o "Patrimonio Consolidado" cae drásticamente en comparación con la instantánea de la semana pasada, podría generar una alerta.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5. Reportes Históricos en PDF:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> Podrías generar un reporte automático que te muestre la evolución patrimonial de todo un año fiscal, ideal para declaraciones o cierres contables.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>6. Análisis de Composición del Portafolio:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> Guardando también los datos de "Distribución de Capital", podrás ver en un gráfico de áreas apiladas cómo ha ido cambiando tu perfil de riesgo con el tiempo (por ejemplo, ver cómo pasaste de tener 80% en Renta Fija a 60% Renta Fija y 40% Acciones a lo largo de 3 años).</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -196,8 +337,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="7"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -207,6 +362,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -238,7 +399,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -253,6 +414,18 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -276,13 +449,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -372,14 +545,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>68035</xdr:colOff>
-      <xdr:row>30</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>76541</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>3925178</xdr:colOff>
-      <xdr:row>48</xdr:row>
-      <xdr:rowOff>80202</xdr:rowOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>80203</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -679,7 +852,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
@@ -1173,12 +1346,14 @@
         <v>1</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F22" s="3">
         <v>46249</v>
       </c>
-      <c r="G22" s="2"/>
+      <c r="G22" s="3">
+        <v>46250</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
@@ -1194,12 +1369,14 @@
         <v>1</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F23" s="3">
         <v>46249</v>
       </c>
-      <c r="G23" s="2"/>
+      <c r="G23" s="3">
+        <v>46250</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -1285,63 +1462,147 @@
       </c>
       <c r="G27" s="2"/>
     </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C28" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C29" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E30">
+      <c r="C30" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C31" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C32" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C33" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C34" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C35" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C36" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C37" s="8"/>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C38" s="8"/>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C39" s="8"/>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C40" s="8"/>
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C41" s="8"/>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C42" s="8"/>
+    </row>
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C43" s="8"/>
+    </row>
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C44" s="8"/>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C45" s="8"/>
+    </row>
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C46" s="8"/>
+    </row>
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C47" s="8"/>
+    </row>
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C48" s="8"/>
+    </row>
+    <row r="49" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C49" s="8"/>
+    </row>
+    <row r="51" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E51">
         <v>28401.05</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C31"/>
-      <c r="E31" s="7">
+    <row r="52" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C52"/>
+      <c r="E52" s="7">
         <v>28374.3</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E32">
-        <f>E30-E31</f>
+    <row r="53" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E53">
+        <f>E51-E52</f>
         <v>26.75</v>
       </c>
     </row>
-    <row r="37" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E37" t="s">
+    <row r="58" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E58" t="s">
         <v>44</v>
       </c>
-      <c r="F37">
+      <c r="F58">
         <v>696</v>
       </c>
     </row>
-    <row r="38" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E38" t="s">
+    <row r="59" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E59" t="s">
         <v>45</v>
       </c>
-      <c r="F38">
+      <c r="F59">
         <v>146</v>
       </c>
     </row>
-    <row r="41" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E41">
+    <row r="62" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E62">
         <v>752.79</v>
       </c>
-      <c r="F41">
+      <c r="F62">
         <v>26.75</v>
       </c>
     </row>
-    <row r="42" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E42">
+    <row r="63" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E63">
         <v>100</v>
       </c>
-      <c r="F42">
-        <f>E42*F41/E41</f>
+      <c r="F63">
+        <f>E63*F62/E62</f>
         <v>3.5534478406992656</v>
       </c>
     </row>
-    <row r="47" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C47" s="6" t="s">
+    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C68" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C49" s="6" t="s">
+    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C70" s="6" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adicion de campo valor nominal en ventas renta fija
</commit_message>
<xml_diff>
--- a/documentacion/TO_DO.xlsx
+++ b/documentacion/TO_DO.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC92654-0AED-4DD8-92BC-34E30F2F5E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE1CA01-F9A8-48D3-AD09-80184BA399B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$27</definedName>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="58">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -315,6 +316,9 @@
       </rPr>
       <t> Guardando también los datos de "Distribución de Capital", podrás ver en un gráfico de áreas apiladas cómo ha ido cambiando tu perfil de riesgo con el tiempo (por ejemplo, ver cómo pasaste de tener 80% en Renta Fija a 60% Renta Fija y 40% Acciones a lo largo de 3 años).</t>
     </r>
+  </si>
+  <si>
+    <t>La funcionalidad de notas de crédito debe cambiarse, no necesitamos la amortizacion</t>
   </si>
 </sst>
 </file>
@@ -372,7 +376,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -395,11 +399,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -426,6 +441,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -496,54 +512,6 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1026" name="AutoShape 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C84F955B-FE31-4790-B273-2F6834EAA456}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr>
-          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvSpPr>
-      </xdr:nvSpPr>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="1181100" y="3619500"/>
-          <a:ext cx="304800" cy="304800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
       <xdr:colOff>68035</xdr:colOff>
       <xdr:row>51</xdr:row>
       <xdr:rowOff>76541</xdr:rowOff>
@@ -585,6 +553,54 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="301398"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CC6E37B-FEAE-402D-AA91-515035F6A5D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="1181100" y="2857500"/>
+          <a:ext cx="304800" cy="301398"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1237,12 +1253,14 @@
         <v>1</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F17" s="3">
         <v>46204</v>
       </c>
-      <c r="G17" s="2"/>
+      <c r="G17" s="3">
+        <v>46256</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
@@ -1463,88 +1481,24 @@
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C28" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C29" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C30" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C31" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C32" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C33" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C34" s="11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C35" s="11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C36" s="11" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C37" s="8"/>
-    </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C38" s="8"/>
-    </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C39" s="8"/>
-    </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C40" s="8"/>
-    </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C41" s="8"/>
-    </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C42" s="8"/>
-    </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C43" s="8"/>
-    </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C44" s="8"/>
-    </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C45" s="8"/>
-    </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C46" s="8"/>
-    </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C47" s="8"/>
-    </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C48" s="8"/>
-    </row>
-    <row r="49" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C49" s="8"/>
+      <c r="A28" s="12">
+        <v>27</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="2">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="3">
+        <v>46255</v>
+      </c>
     </row>
     <row r="51" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E51">
@@ -1617,4 +1571,99 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8D89EDA-31BE-4A34-91D4-C557DE541979}">
+  <dimension ref="C2:C23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="3:3" ht="135" x14ac:dyDescent="0.25">
+      <c r="C2" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C5" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C6" s="11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C7" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C8" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C9" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C10" s="11" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C11" s="8"/>
+    </row>
+    <row r="12" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="8"/>
+    </row>
+    <row r="13" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C13" s="8"/>
+    </row>
+    <row r="14" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C14" s="8"/>
+    </row>
+    <row r="15" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="8"/>
+    </row>
+    <row r="16" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C16" s="8"/>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C17" s="8"/>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C18" s="8"/>
+    </row>
+    <row r="19" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C19" s="8"/>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="8"/>
+    </row>
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C21" s="8"/>
+    </row>
+    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C22" s="8"/>
+    </row>
+    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>